<commit_message>
actualzacion 25/08/2025 21:55 disparador
</commit_message>
<xml_diff>
--- a/02.descargable/XLSX/01.XLSX correctos/reseñas.xlsx
+++ b/02.descargable/XLSX/01.XLSX correctos/reseñas.xlsx
@@ -472,12 +472,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>C-001531</t>
+          <t>C-002124</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CL-05513</t>
+          <t>CL-02665</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -485,11 +485,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>45889</v>
+        <v>45867</v>
       </c>
     </row>
     <row r="3">
@@ -500,24 +500,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C-000291</t>
+          <t>C-001960</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CL-02529</t>
+          <t>CL-09251</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>45859</v>
+        <v>45881</v>
       </c>
     </row>
     <row r="4">
@@ -528,24 +528,24 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C-001221</t>
+          <t>C-001614</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CL-01649</t>
+          <t>CL-04714</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>45851</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="5">
@@ -556,12 +556,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C-001760</t>
+          <t>C-001036</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CL-05951</t>
+          <t>CL-04811</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -569,11 +569,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>45882</v>
+        <v>45875</v>
       </c>
     </row>
     <row r="6">
@@ -584,24 +584,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>C-000752</t>
+          <t>C-004127</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CL-04106</t>
+          <t>CL-02695</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>45866</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="7">
@@ -612,24 +612,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>C-002352</t>
+          <t>C-003433</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CL-02900</t>
+          <t>CL-05872</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>45866</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="8">
@@ -640,16 +640,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>C-002756</t>
+          <t>C-002951</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CL-05673</t>
+          <t>CL-06266</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>45851</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="9">
@@ -668,20 +668,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>C-004561</t>
+          <t>C-001950</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CL-07335</t>
+          <t>CL-01372</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -696,24 +696,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>C-004025</t>
+          <t>C-003244</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CL-01907</t>
+          <t>CL-02948</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>45867</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="11">
@@ -724,24 +724,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>C-001563</t>
+          <t>C-004767</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CL-05770</t>
+          <t>CL-03797</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>45869</v>
+        <v>45826</v>
       </c>
     </row>
     <row r="12">
@@ -752,12 +752,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>C-003004</t>
+          <t>C-000132</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CL-08389</t>
+          <t>CL-06301</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -765,11 +765,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>45844</v>
+        <v>45857</v>
       </c>
     </row>
     <row r="13">
@@ -780,12 +780,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C-004855</t>
+          <t>C-002116</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CL-05023</t>
+          <t>CL-09738</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -793,11 +793,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Todo perfecto, gracias.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>45890</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="14">
@@ -808,16 +808,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C-001289</t>
+          <t>C-002943</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CL-03861</t>
+          <t>CL-09329</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>45832</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="15">
@@ -836,12 +836,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C-002931</t>
+          <t>C-002895</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>CL-04253</t>
+          <t>CL-02576</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -849,11 +849,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>45872</v>
+        <v>45885</v>
       </c>
     </row>
     <row r="16">
@@ -864,24 +864,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C-001078</t>
+          <t>C-001198</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CL-09696</t>
+          <t>CL-05261</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>El embalaje estaba dañado.</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>45828</v>
+        <v>45863</v>
       </c>
     </row>
     <row r="17">
@@ -892,24 +892,24 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C-000366</t>
+          <t>C-003711</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CL-06730</t>
+          <t>CL-08995</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>45888</v>
+        <v>45890</v>
       </c>
     </row>
     <row r="18">
@@ -920,24 +920,24 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C-000337</t>
+          <t>C-004581</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CL-08441</t>
+          <t>CL-06550</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tuve problemas con la entrega.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>45846</v>
+        <v>45832</v>
       </c>
     </row>
     <row r="19">
@@ -948,24 +948,24 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>C-002730</t>
+          <t>C-004573</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CL-05065</t>
+          <t>CL-04994</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>45853</v>
+        <v>45871</v>
       </c>
     </row>
     <row r="20">
@@ -976,24 +976,24 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>C-000611</t>
+          <t>C-000871</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CL-08139</t>
+          <t>CL-05432</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>El embalaje estaba dañado.</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>45876</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="21">
@@ -1004,24 +1004,24 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>C-002700</t>
+          <t>C-004480</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CL-09913</t>
+          <t>CL-04364</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>Me encantó, lo recomiendo.</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>45869</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="22">
@@ -1032,24 +1032,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>C-002490</t>
+          <t>C-002818</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CL-06599</t>
+          <t>CL-03658</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Todo perfecto, gracias.</t>
+          <t>Me encantó, lo recomiendo.</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>45879</v>
+        <v>45816</v>
       </c>
     </row>
     <row r="23">
@@ -1060,24 +1060,24 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>C-004573</t>
+          <t>C-001249</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CL-01518</t>
+          <t>CL-08995</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>45879</v>
+        <v>45885</v>
       </c>
     </row>
     <row r="24">
@@ -1088,12 +1088,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>C-003615</t>
+          <t>C-001171</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CL-02749</t>
+          <t>CL-05987</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1101,11 +1101,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>45855</v>
+        <v>45834</v>
       </c>
     </row>
     <row r="25">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C-004319</t>
+          <t>C-002178</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CL-05066</t>
+          <t>CL-06640</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1129,11 +1129,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>45876</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="26">
@@ -1144,12 +1144,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>C-002674</t>
+          <t>C-001195</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CL-05641</t>
+          <t>CL-05139</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1157,11 +1157,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>45892</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="27">
@@ -1172,12 +1172,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C-001849</t>
+          <t>C-003394</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CL-02455</t>
+          <t>CL-05279</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1185,11 +1185,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>45842</v>
+        <v>45839</v>
       </c>
     </row>
     <row r="28">
@@ -1200,12 +1200,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>C-003253</t>
+          <t>C-001770</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CL-09604</t>
+          <t>CL-08883</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1213,11 +1213,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>45879</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="29">
@@ -1228,24 +1228,24 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>C-002550</t>
+          <t>C-000549</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CL-08286</t>
+          <t>CL-04285</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>45881</v>
+        <v>45870</v>
       </c>
     </row>
     <row r="30">
@@ -1256,24 +1256,24 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>C-000179</t>
+          <t>C-003598</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CL-01545</t>
+          <t>CL-03797</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>45881</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="31">
@@ -1284,24 +1284,24 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>C-004899</t>
+          <t>C-002016</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CL-00291</t>
+          <t>CL-07547</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>45858</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="32">
@@ -1312,16 +1312,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>C-001552</t>
+          <t>C-001094</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CL-02886</t>
+          <t>CL-06552</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>45836</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="33">
@@ -1340,12 +1340,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>C-003230</t>
+          <t>C-002154</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CL-09322</t>
+          <t>CL-06245</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1353,11 +1353,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>45888</v>
+        <v>45853</v>
       </c>
     </row>
     <row r="34">
@@ -1368,24 +1368,24 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>C-000864</t>
+          <t>C-003587</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CL-01765</t>
+          <t>CL-00879</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>El embalaje estaba dañado.</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>45892</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="35">
@@ -1396,24 +1396,24 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>C-000751</t>
+          <t>C-004206</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CL-09774</t>
+          <t>CL-07253</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>45864</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="36">
@@ -1424,24 +1424,24 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>C-002046</t>
+          <t>C-004607</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CL-05289</t>
+          <t>CL-06999</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>45892</v>
+        <v>45890</v>
       </c>
     </row>
     <row r="37">
@@ -1452,12 +1452,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>C-000939</t>
+          <t>C-004280</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CL-00715</t>
+          <t>CL-05658</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1465,11 +1465,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>45892</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="38">
@@ -1480,24 +1480,24 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>C-001166</t>
+          <t>C-000435</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CL-05699</t>
+          <t>CL-08952</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>45877</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="39">
@@ -1508,24 +1508,24 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>C-003085</t>
+          <t>C-002436</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CL-08434</t>
+          <t>CL-05159</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>45886</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="40">
@@ -1536,24 +1536,24 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>C-003497</t>
+          <t>C-000370</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CL-06058</t>
+          <t>CL-09478</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Todo perfecto, gracias.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>45856</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="41">
@@ -1564,24 +1564,24 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>C-001787</t>
+          <t>C-004582</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CL-02816</t>
+          <t>CL-06380</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>45835</v>
+        <v>45842</v>
       </c>
     </row>
     <row r="42">
@@ -1592,24 +1592,24 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>C-002542</t>
+          <t>C-004329</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CL-03835</t>
+          <t>CL-03936</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>45884</v>
+        <v>45881</v>
       </c>
     </row>
     <row r="43">
@@ -1620,24 +1620,24 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>C-004801</t>
+          <t>C-003400</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CL-05193</t>
+          <t>CL-01293</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>45869</v>
+        <v>45876</v>
       </c>
     </row>
     <row r="44">
@@ -1648,24 +1648,24 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>C-001011</t>
+          <t>C-000733</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CL-01722</t>
+          <t>CL-05782</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>45892</v>
+        <v>45866</v>
       </c>
     </row>
     <row r="45">
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>C-001108</t>
+          <t>C-001260</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CL-03245</t>
+          <t>CL-09057</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1689,11 +1689,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>45882</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="46">
@@ -1704,24 +1704,24 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>C-003469</t>
+          <t>C-004014</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CL-08773</t>
+          <t>CL-09899</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>45839</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="47">
@@ -1732,24 +1732,24 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>C-002405</t>
+          <t>C-002225</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CL-06087</t>
+          <t>CL-01373</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>45880</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="48">
@@ -1760,24 +1760,24 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>C-004122</t>
+          <t>C-002966</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CL-08221</t>
+          <t>CL-07796</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>45846</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="49">
@@ -1788,24 +1788,24 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C-001488</t>
+          <t>C-004691</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CL-03641</t>
+          <t>CL-06497</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>45858</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="50">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>C-000527</t>
+          <t>C-003198</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CL-03028</t>
+          <t>CL-01140</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>45891</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="51">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>C-003594</t>
+          <t>C-004794</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CL-07854</t>
+          <t>CL-03353</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1857,11 +1857,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>Me encantó, lo recomiendo.</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>45889</v>
+        <v>45866</v>
       </c>
     </row>
     <row r="52">
@@ -1872,16 +1872,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>C-001654</t>
+          <t>C-000552</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CL-01729</t>
+          <t>CL-01352</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>45887</v>
+        <v>45872</v>
       </c>
     </row>
     <row r="53">
@@ -1900,24 +1900,24 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>C-003580</t>
+          <t>C-003377</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CL-09301</t>
+          <t>CL-00092</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>45871</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="54">
@@ -1928,24 +1928,24 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>C-001028</t>
+          <t>C-003843</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CL-07341</t>
+          <t>CL-05578</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>45887</v>
+        <v>45883</v>
       </c>
     </row>
     <row r="55">
@@ -1956,24 +1956,24 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>C-002679</t>
+          <t>C-001709</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CL-07068</t>
+          <t>CL-00215</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>45811</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="56">
@@ -1984,24 +1984,24 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>C-002900</t>
+          <t>C-003971</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CL-00839</t>
+          <t>CL-04712</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>45885</v>
+        <v>45834</v>
       </c>
     </row>
     <row r="57">
@@ -2012,24 +2012,24 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>C-003202</t>
+          <t>C-000112</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CL-07955</t>
+          <t>CL-09223</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>45888</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="58">
@@ -2040,12 +2040,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>C-003940</t>
+          <t>C-003454</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CL-01377</t>
+          <t>CL-07302</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2053,11 +2053,11 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>45861</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="59">
@@ -2068,24 +2068,24 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>C-001244</t>
+          <t>C-002233</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CL-04645</t>
+          <t>CL-03239</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Todo perfecto, gracias.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>45835</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="60">
@@ -2096,24 +2096,24 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>C-003363</t>
+          <t>C-004555</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CL-06142</t>
+          <t>CL-08016</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>45880</v>
+        <v>45846</v>
       </c>
     </row>
     <row r="61">
@@ -2124,24 +2124,24 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>C-001451</t>
+          <t>C-003248</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>CL-03402</t>
+          <t>CL-03795</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>45843</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="62">
@@ -2152,24 +2152,24 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>C-000705</t>
+          <t>C-003315</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CL-06792</t>
+          <t>CL-04813</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Tuve problemas con la entrega.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>45892</v>
+        <v>45887</v>
       </c>
     </row>
     <row r="63">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>C-000469</t>
+          <t>C-001957</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>CL-09450</t>
+          <t>CL-01550</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -2193,11 +2193,11 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>45863</v>
+        <v>45891</v>
       </c>
     </row>
     <row r="64">
@@ -2208,12 +2208,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>C-003535</t>
+          <t>C-001526</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CL-04452</t>
+          <t>CL-08716</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2221,11 +2221,11 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>45874</v>
+        <v>45854</v>
       </c>
     </row>
     <row r="65">
@@ -2236,12 +2236,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>C-000830</t>
+          <t>C-001444</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CL-08829</t>
+          <t>CL-01451</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>45884</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="66">
@@ -2264,24 +2264,24 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>C-003508</t>
+          <t>C-002656</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>CL-01494</t>
+          <t>CL-09528</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>45873</v>
+        <v>45893</v>
       </c>
     </row>
     <row r="67">
@@ -2292,24 +2292,24 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>C-001361</t>
+          <t>C-004041</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CL-02515</t>
+          <t>CL-07504</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>45871</v>
+        <v>45878</v>
       </c>
     </row>
     <row r="68">
@@ -2320,24 +2320,24 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>C-001519</t>
+          <t>C-002394</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CL-06912</t>
+          <t>CL-09129</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>45878</v>
+        <v>45828</v>
       </c>
     </row>
     <row r="69">
@@ -2348,24 +2348,24 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>C-002007</t>
+          <t>C-000875</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CL-07749</t>
+          <t>CL-05564</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>45873</v>
+        <v>45892</v>
       </c>
     </row>
     <row r="70">
@@ -2376,12 +2376,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>C-002844</t>
+          <t>C-000640</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CL-09295</t>
+          <t>CL-05975</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2389,11 +2389,11 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>El embalaje estaba dañado.</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>45870</v>
+        <v>45874</v>
       </c>
     </row>
     <row r="71">
@@ -2404,12 +2404,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>C-004945</t>
+          <t>C-004207</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CL-02578</t>
+          <t>CL-03355</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>45847</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="72">
@@ -2432,24 +2432,24 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>C-002204</t>
+          <t>C-001905</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CL-07621</t>
+          <t>CL-02031</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>El embalaje estaba dañado.</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>45861</v>
+        <v>45869</v>
       </c>
     </row>
     <row r="73">
@@ -2460,24 +2460,24 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>C-003923</t>
+          <t>C-002238</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CL-00965</t>
+          <t>CL-05678</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>45891</v>
+        <v>45827</v>
       </c>
     </row>
     <row r="74">
@@ -2488,24 +2488,24 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>C-004652</t>
+          <t>C-001992</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>CL-04033</t>
+          <t>CL-03825</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>45890</v>
+        <v>45837</v>
       </c>
     </row>
     <row r="75">
@@ -2516,12 +2516,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>C-004922</t>
+          <t>C-001781</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>CL-09867</t>
+          <t>CL-08664</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2529,11 +2529,11 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>45876</v>
+        <v>45883</v>
       </c>
     </row>
     <row r="76">
@@ -2544,12 +2544,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>C-004498</t>
+          <t>C-003132</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CL-01368</t>
+          <t>CL-04683</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2557,11 +2557,11 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Me encantó, lo recomiendo.</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>45874</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="77">
@@ -2572,12 +2572,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>C-001883</t>
+          <t>C-003561</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CL-06660</t>
+          <t>CL-09251</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2585,11 +2585,11 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Tuve problemas con la entrega.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>45872</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="78">
@@ -2600,24 +2600,24 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>C-002354</t>
+          <t>C-002958</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>CL-09388</t>
+          <t>CL-07956</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>45866</v>
+        <v>45841</v>
       </c>
     </row>
     <row r="79">
@@ -2628,24 +2628,24 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>C-000648</t>
+          <t>C-001856</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CL-06984</t>
+          <t>CL-00861</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>45878</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="80">
@@ -2656,24 +2656,24 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>C-001645</t>
+          <t>C-001103</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>CL-01734</t>
+          <t>CL-00956</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Excelente atención al cliente.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>45868</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="81">
@@ -2684,16 +2684,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>C-003412</t>
+          <t>C-004826</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CL-00746</t>
+          <t>CL-09892</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2701,7 +2701,7 @@
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>45875</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="82">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>C-000196</t>
+          <t>C-003025</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CL-04467</t>
+          <t>CL-09547</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2725,11 +2725,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>45869</v>
+        <v>45848</v>
       </c>
     </row>
     <row r="83">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>C-002432</t>
+          <t>C-000579</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CL-02989</t>
+          <t>CL-03733</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2753,11 +2753,11 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Todo perfecto, gracias.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>45888</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="84">
@@ -2768,24 +2768,24 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>C-004035</t>
+          <t>C-001410</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CL-02340</t>
+          <t>CL-02577</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Todo perfecto, gracias.</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
-        <v>45853</v>
+        <v>45880</v>
       </c>
     </row>
     <row r="85">
@@ -2796,24 +2796,24 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>C-000707</t>
+          <t>C-002973</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>CL-00080</t>
+          <t>CL-05884</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Tuve problemas con la entrega.</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>45867</v>
+        <v>45850</v>
       </c>
     </row>
     <row r="86">
@@ -2824,12 +2824,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>C-001136</t>
+          <t>C-001527</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CL-09780</t>
+          <t>CL-05487</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2837,11 +2837,11 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Todo perfecto, gracias.</t>
+          <t>Precio justo y buena calidad.</t>
         </is>
       </c>
       <c r="F86" s="2" t="n">
-        <v>45848</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="87">
@@ -2852,16 +2852,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>C-000191</t>
+          <t>C-001408</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CL-06860</t>
+          <t>CL-03514</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>45879</v>
+        <v>45837</v>
       </c>
     </row>
     <row r="88">
@@ -2880,16 +2880,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>C-004958</t>
+          <t>C-004830</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CL-05231</t>
+          <t>CL-06380</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2897,7 +2897,7 @@
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>45866</v>
+        <v>45858</v>
       </c>
     </row>
     <row r="89">
@@ -2908,24 +2908,24 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>C-004291</t>
+          <t>C-002047</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>CL-04178</t>
+          <t>CL-09732</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F89" s="2" t="n">
-        <v>45873</v>
+        <v>45854</v>
       </c>
     </row>
     <row r="90">
@@ -2936,16 +2936,16 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>C-000685</t>
+          <t>C-000578</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>CL-00136</t>
+          <t>CL-06738</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2953,7 +2953,7 @@
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>45886</v>
+        <v>45856</v>
       </c>
     </row>
     <row r="91">
@@ -2964,12 +2964,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>C-002932</t>
+          <t>C-003660</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CL-08041</t>
+          <t>CL-03736</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="F91" s="2" t="n">
-        <v>45858</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="92">
@@ -2992,12 +2992,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>C-002434</t>
+          <t>C-003516</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CL-05886</t>
+          <t>CL-03576</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -3005,11 +3005,11 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>La talla no era correcta.</t>
+          <t>No era lo que esperaba.</t>
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>45883</v>
+        <v>45881</v>
       </c>
     </row>
     <row r="93">
@@ -3020,24 +3020,24 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>C-003415</t>
+          <t>C-000376</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>CL-05645</t>
+          <t>CL-05701</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>La talla no era correcta.</t>
         </is>
       </c>
       <c r="F93" s="2" t="n">
-        <v>45887</v>
+        <v>45877</v>
       </c>
     </row>
     <row r="94">
@@ -3048,16 +3048,16 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>C-004651</t>
+          <t>C-003985</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>CL-06335</t>
+          <t>CL-06413</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -3065,7 +3065,7 @@
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>45847</v>
+        <v>45855</v>
       </c>
     </row>
     <row r="95">
@@ -3076,12 +3076,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>C-000766</t>
+          <t>C-003235</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>CL-09380</t>
+          <t>CL-02809</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -3089,11 +3089,11 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Precio justo y buena calidad.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F95" s="2" t="n">
-        <v>45892</v>
+        <v>45859</v>
       </c>
     </row>
     <row r="96">
@@ -3104,24 +3104,24 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>C-003296</t>
+          <t>C-000647</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>CL-01165</t>
+          <t>CL-05576</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Volveré a comprar sin duda.</t>
+          <t>Muy buen producto, llegó rápido.</t>
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>45854</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="97">
@@ -3132,24 +3132,24 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>C-003297</t>
+          <t>C-004162</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>CL-00221</t>
+          <t>CL-07648</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>El embalaje estaba dañado.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F97" s="2" t="n">
-        <v>45875</v>
+        <v>45886</v>
       </c>
     </row>
     <row r="98">
@@ -3160,12 +3160,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>C-002023</t>
+          <t>C-002748</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>CL-09962</t>
+          <t>CL-01544</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -3173,11 +3173,11 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Me encantó, lo recomiendo.</t>
         </is>
       </c>
       <c r="F98" s="2" t="n">
-        <v>45885</v>
+        <v>45884</v>
       </c>
     </row>
     <row r="99">
@@ -3188,24 +3188,24 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>C-001431</t>
+          <t>C-002520</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>CL-06350</t>
+          <t>CL-02161</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Muy buen producto, llegó rápido.</t>
+          <t>Volveré a comprar sin duda.</t>
         </is>
       </c>
       <c r="F99" s="2" t="n">
-        <v>45871</v>
+        <v>45818</v>
       </c>
     </row>
     <row r="100">
@@ -3216,12 +3216,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>C-003811</t>
+          <t>C-004249</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CL-00101</t>
+          <t>CL-07039</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3229,11 +3229,11 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Me encantó, lo recomiendo.</t>
+          <t>El embalaje estaba dañado.</t>
         </is>
       </c>
       <c r="F100" s="2" t="n">
-        <v>45865</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="101">
@@ -3244,12 +3244,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>C-003287</t>
+          <t>C-004393</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CL-00179</t>
+          <t>CL-08090</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -3257,11 +3257,11 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>No era lo que esperaba.</t>
+          <t>Excelente atención al cliente.</t>
         </is>
       </c>
       <c r="F101" s="2" t="n">
-        <v>45839</v>
+        <v>45868</v>
       </c>
     </row>
   </sheetData>

</xml_diff>